<commit_message>
read kernel from disk part 1
</commit_message>
<xml_diff>
--- a/res/ram-memory.xlsx
+++ b/res/ram-memory.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="tZn3PkswWhaNE9w/WeFbyxDEICZ7EZH5QH9sB2nWxo8="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="X3FWWEs0pVGbOJ+1wR3jKmyUr8Kcw4rF7S1X3S2Hfs0="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>0 KB</t>
   </si>
@@ -253,6 +253,29 @@
   </si>
   <si>
     <t>112 KB</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+        <sz val="9.0"/>
+      </rPr>
+      <t>112 KB — 116 KB</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="11.0"/>
+      </rPr>
+      <t xml:space="preserve">
+E820 Map</t>
+    </r>
+  </si>
+  <si>
+    <t>116 KB</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -1113,11 +1136,11 @@
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
     </row>
-    <row r="11" ht="394.5" customHeight="1">
+    <row r="11" ht="37.5" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="7" t="s">
         <v>22</v>
       </c>
       <c r="C11" s="3"/>
@@ -1145,11 +1168,11 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" s="1" t="s">
+    <row r="12" ht="394.5" customHeight="1">
+      <c r="A12" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="11" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="3"/>
@@ -1177,11 +1200,11 @@
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
     </row>
-    <row r="13" ht="43.5" customHeight="1">
+    <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="3"/>
@@ -1209,7 +1232,7 @@
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
     </row>
-    <row r="14" ht="37.5" customHeight="1">
+    <row r="14" ht="43.5" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>27</v>
       </c>
@@ -1241,11 +1264,11 @@
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
     </row>
-    <row r="15" ht="49.5" customHeight="1">
+    <row r="15" ht="37.5" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="12" t="s">
         <v>30</v>
       </c>
       <c r="C15" s="3"/>
@@ -1273,11 +1296,11 @@
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
     </row>
-    <row r="16" ht="61.5" customHeight="1">
+    <row r="16" ht="49.5" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C16" s="3"/>
@@ -1305,11 +1328,11 @@
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
     </row>
-    <row r="17" ht="36.0" customHeight="1">
+    <row r="17" ht="61.5" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="12" t="s">
         <v>34</v>
       </c>
       <c r="C17" s="3"/>
@@ -1337,7 +1360,7 @@
       <c r="Y17" s="3"/>
       <c r="Z17" s="3"/>
     </row>
-    <row r="18" ht="39.75" customHeight="1">
+    <row r="18" ht="36.0" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
@@ -1369,11 +1392,11 @@
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
     </row>
-    <row r="19" ht="409.5" customHeight="1">
+    <row r="19" ht="39.75" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="3"/>
@@ -1401,9 +1424,13 @@
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
     </row>
-    <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+    <row r="20" ht="409.5" customHeight="1">
+      <c r="A20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -29037,6 +29064,34 @@
       <c r="Y1006" s="3"/>
       <c r="Z1006" s="3"/>
     </row>
+    <row r="1007" ht="14.25" customHeight="1">
+      <c r="A1007" s="3"/>
+      <c r="B1007" s="3"/>
+      <c r="C1007" s="3"/>
+      <c r="D1007" s="3"/>
+      <c r="E1007" s="3"/>
+      <c r="F1007" s="3"/>
+      <c r="G1007" s="3"/>
+      <c r="H1007" s="3"/>
+      <c r="I1007" s="3"/>
+      <c r="J1007" s="3"/>
+      <c r="K1007" s="3"/>
+      <c r="L1007" s="3"/>
+      <c r="M1007" s="3"/>
+      <c r="N1007" s="3"/>
+      <c r="O1007" s="3"/>
+      <c r="P1007" s="3"/>
+      <c r="Q1007" s="3"/>
+      <c r="R1007" s="3"/>
+      <c r="S1007" s="3"/>
+      <c r="T1007" s="3"/>
+      <c r="U1007" s="3"/>
+      <c r="V1007" s="3"/>
+      <c r="W1007" s="3"/>
+      <c r="X1007" s="3"/>
+      <c r="Y1007" s="3"/>
+      <c r="Z1007" s="3"/>
+    </row>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>